<commit_message>
Simplify PriceSpider widget; settings move to page metadata
- where-to-buy.js: only builds the .ps-widget mount and loads ps-widget.js
  and ps-utid.js; ps-* account settings now come from page metadata and
  PriceSpider reads ?ps-sku= itself (matches production)
- where-to-buy.css: drop fallback message styles
- importer: copy ps-* meta tags from the source page into page metadata

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-where-to-buy.report.xlsx
+++ b/tools/importer/reports/import-where-to-buy.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
   <si>
     <t>_reportFile</t>
   </si>
@@ -55,7 +55,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-15T17:37:54.387Z</t>
+    <t>2026-10-18T18:31:05.924Z</t>
   </si>
   <si>
     <t>Where to Buy</t>
@@ -104,6 +104,30 @@
   </si>
   <si>
     <t>https://www.hersheyland.com/products/reeses-oreo-milk-chocolate-peanut-butter-cups-1-4-oz.html</t>
+  </si>
+  <si>
+    <t>recipes/reeses-oreo-cup-brownies.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb-trail","hero-recipe","columns-recipe","fragment","cards-recipe","columns-nutrition","widget"]</t>
+  </si>
+  <si>
+    <t>990</t>
+  </si>
+  <si>
+    <t>recipes/reeses-oreo-cup-brownies</t>
+  </si>
+  <si>
+    <t>recipe-detail</t>
+  </si>
+  <si>
+    <t>2026-10-15T11:39:27.870Z</t>
+  </si>
+  <si>
+    <t>REESE’S OREO® Cup Brownies</t>
+  </si>
+  <si>
+    <t>https://www.hersheyland.com/recipes/reeses-oreo-cup-brownies.html</t>
   </si>
 </sst>
 </file>
@@ -492,13 +516,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="50" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="9" width="50" customWidth="1"/>
   </cols>
@@ -619,6 +643,35 @@
         <v>30</v>
       </c>
     </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>